<commit_message>
charts styling / sorting / reimport past data
</commit_message>
<xml_diff>
--- a/planing/sample.xlsx
+++ b/planing/sample.xlsx
@@ -411,7 +411,7 @@
     </row>
     <row r="2">
       <c r="A2" s="9">
-        <v>45658.0</v>
+        <v>45657.0</v>
       </c>
       <c r="B2" s="10">
         <v>19.102</v>
@@ -437,7 +437,7 @@
     </row>
     <row r="3">
       <c r="A3" s="9">
-        <v>45689.0</v>
+        <v>45688.0</v>
       </c>
       <c r="B3" s="10">
         <v>22.75</v>
@@ -463,7 +463,7 @@
     </row>
     <row r="4">
       <c r="A4" s="9">
-        <v>45720.0</v>
+        <v>45716.0</v>
       </c>
       <c r="B4" s="10">
         <v>26.1</v>
@@ -515,7 +515,7 @@
     </row>
     <row r="6">
       <c r="A6" s="9">
-        <v>45784.0</v>
+        <v>45777.0</v>
       </c>
       <c r="B6" s="10">
         <v>35.31</v>
@@ -541,7 +541,7 @@
     </row>
     <row r="7">
       <c r="A7" s="9">
-        <v>45810.0</v>
+        <v>45808.0</v>
       </c>
       <c r="B7" s="10">
         <v>39.18</v>
@@ -568,7 +568,7 @@
     </row>
     <row r="8">
       <c r="A8" s="9">
-        <v>45842.0</v>
+        <v>45838.0</v>
       </c>
       <c r="B8" s="10">
         <v>43.8</v>
@@ -595,7 +595,7 @@
     </row>
     <row r="9">
       <c r="A9" s="9">
-        <v>45881.0</v>
+        <v>45869.0</v>
       </c>
       <c r="B9" s="10">
         <v>49.7</v>
@@ -622,7 +622,7 @@
     </row>
     <row r="10">
       <c r="A10" s="9">
-        <v>45906.0</v>
+        <v>45900.0</v>
       </c>
       <c r="B10" s="10">
         <v>53.67</v>
@@ -649,7 +649,7 @@
     </row>
     <row r="11">
       <c r="A11" s="9">
-        <v>45931.0</v>
+        <v>45930.0</v>
       </c>
       <c r="B11" s="10">
         <v>58.3</v>
@@ -676,7 +676,7 @@
     </row>
     <row r="12">
       <c r="A12" s="9">
-        <v>45964.0</v>
+        <v>45961.0</v>
       </c>
       <c r="B12" s="10">
         <v>62.48</v>
@@ -703,7 +703,7 @@
     </row>
     <row r="13">
       <c r="A13" s="9">
-        <v>45992.0</v>
+        <v>45991.0</v>
       </c>
       <c r="B13" s="10">
         <v>65.08</v>

</xml_diff>